<commit_message>
banking website test scripts
</commit_message>
<xml_diff>
--- a/Banking test cases.xlsx
+++ b/Banking test cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\OneDrive\Desktop\Banking test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B58559D8-E525-48D3-A480-A09E4426B9CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BC974FB-D53D-4ABF-A71E-B62E3E1AD7BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -95,16 +95,7 @@
     <t>Opening existed customer details with valid ID</t>
   </si>
   <si>
-    <t xml:space="preserve">Opening with invalid ID </t>
-  </si>
-  <si>
     <t xml:space="preserve">Deleting Customer </t>
-  </si>
-  <si>
-    <t xml:space="preserve">with valid ID </t>
-  </si>
-  <si>
-    <t>With invalid ID</t>
   </si>
   <si>
     <t>Add new account Page</t>
@@ -219,6 +210,15 @@
   </si>
   <si>
     <t>redirecting to home page</t>
+  </si>
+  <si>
+    <t>with valid ID</t>
+  </si>
+  <si>
+    <t>With invalid ID and black data</t>
+  </si>
+  <si>
+    <t>Opening with invalid ID, blank id</t>
   </si>
 </sst>
 </file>
@@ -516,7 +516,7 @@
   <dimension ref="A1:Z1000"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="145.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1216,7 +1216,7 @@
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1" t="s">
-        <v>24</v>
+        <v>65</v>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
@@ -1273,10 +1273,10 @@
     <row r="26" spans="1:26" ht="14.25">
       <c r="A26" s="1"/>
       <c r="B26" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>26</v>
+        <v>63</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
@@ -1306,7 +1306,7 @@
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1" t="s">
-        <v>27</v>
+        <v>64</v>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
@@ -1363,10 +1363,10 @@
     <row r="29" spans="1:26" ht="14.25">
       <c r="A29" s="1"/>
       <c r="B29" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
@@ -1396,7 +1396,7 @@
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
@@ -1426,7 +1426,7 @@
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
@@ -1456,7 +1456,7 @@
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
@@ -1486,7 +1486,7 @@
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
@@ -1516,7 +1516,7 @@
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
@@ -1546,7 +1546,7 @@
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
@@ -1603,10 +1603,10 @@
     <row r="37" spans="1:26" ht="14.25">
       <c r="A37" s="1"/>
       <c r="B37" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D37" s="1"/>
       <c r="E37" s="1"/>
@@ -1636,7 +1636,7 @@
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D38" s="1"/>
       <c r="E38" s="1"/>
@@ -1666,7 +1666,7 @@
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D39" s="1"/>
       <c r="E39" s="1"/>
@@ -1723,10 +1723,10 @@
     <row r="41" spans="1:26" ht="14.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D41" s="1"/>
       <c r="E41" s="1"/>
@@ -1756,7 +1756,7 @@
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D42" s="1"/>
       <c r="E42" s="1"/>
@@ -1786,7 +1786,7 @@
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D43" s="1"/>
       <c r="E43" s="1"/>
@@ -1816,7 +1816,7 @@
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D44" s="1"/>
       <c r="E44" s="1"/>
@@ -1873,10 +1873,10 @@
     <row r="46" spans="1:26" ht="14.25">
       <c r="A46" s="1"/>
       <c r="B46" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D46" s="1"/>
       <c r="E46" s="1"/>
@@ -1906,7 +1906,7 @@
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D47" s="1"/>
       <c r="E47" s="1"/>
@@ -1936,7 +1936,7 @@
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D48" s="1"/>
       <c r="E48" s="1"/>
@@ -1966,7 +1966,7 @@
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D49" s="1"/>
       <c r="E49" s="1"/>
@@ -2023,10 +2023,10 @@
     <row r="51" spans="1:26" ht="14.25">
       <c r="A51" s="1"/>
       <c r="B51" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D51" s="1"/>
       <c r="E51" s="1"/>
@@ -2056,7 +2056,7 @@
       <c r="A52" s="1"/>
       <c r="B52" s="1"/>
       <c r="C52" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D52" s="1"/>
       <c r="E52" s="1"/>
@@ -2086,7 +2086,7 @@
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
       <c r="C53" s="1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D53" s="1"/>
       <c r="E53" s="1"/>
@@ -2116,7 +2116,7 @@
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
       <c r="C54" s="1" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D54" s="1"/>
       <c r="E54" s="1"/>
@@ -2146,7 +2146,7 @@
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
       <c r="C55" s="1" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D55" s="1"/>
       <c r="E55" s="1"/>
@@ -2176,7 +2176,7 @@
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
       <c r="C56" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D56" s="1"/>
       <c r="E56" s="1"/>
@@ -2206,7 +2206,7 @@
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
       <c r="C57" s="1" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D57" s="1"/>
       <c r="E57" s="1"/>
@@ -2236,7 +2236,7 @@
       <c r="A58" s="1"/>
       <c r="B58" s="1"/>
       <c r="C58" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D58" s="1"/>
       <c r="E58" s="1"/>
@@ -2266,7 +2266,7 @@
       <c r="A59" s="1"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D59" s="1"/>
       <c r="E59" s="1"/>
@@ -2296,7 +2296,7 @@
       <c r="A60" s="1"/>
       <c r="B60" s="1"/>
       <c r="C60" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D60" s="1"/>
       <c r="E60" s="1"/>
@@ -2326,7 +2326,7 @@
       <c r="A61" s="1"/>
       <c r="B61" s="1"/>
       <c r="C61" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D61" s="1"/>
       <c r="E61" s="1"/>
@@ -2356,7 +2356,7 @@
       <c r="A62" s="1"/>
       <c r="B62" s="1"/>
       <c r="C62" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D62" s="1"/>
       <c r="E62" s="1"/>
@@ -2386,7 +2386,7 @@
       <c r="A63" s="1"/>
       <c r="B63" s="1"/>
       <c r="C63" s="1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D63" s="1"/>
       <c r="E63" s="1"/>
@@ -2443,10 +2443,10 @@
     <row r="65" spans="1:26" ht="14.25">
       <c r="A65" s="1"/>
       <c r="B65" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D65" s="1"/>
       <c r="E65" s="1"/>

</xml_diff>